<commit_message>
feat(import): add priority conversion with live preview, adjust panel, and confirmation
</commit_message>
<xml_diff>
--- a/samples/sample-leads.xlsx
+++ b/samples/sample-leads.xlsx
@@ -445,34 +445,34 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Sri Krishna Silks</v>
+        <v>Lead Priority Score 0</v>
       </c>
       <c r="B2" t="str">
-        <v>9840123456</v>
+        <v>9840000000</v>
       </c>
       <c r="C2" t="str">
-        <v>contact@krishnasilks.com</v>
+        <v>score0@example.com</v>
       </c>
       <c r="D2" t="str">
-        <v>https://krishnasilks.com</v>
+        <v/>
       </c>
       <c r="E2" t="str">
-        <v>Silk store</v>
+        <v>Boutique</v>
       </c>
       <c r="F2" t="str">
-        <v>14, Gandhi Road, Vellore, Tamil Nadu 632004</v>
+        <v>100 Test St, Vellore</v>
       </c>
       <c r="G2">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="I2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="str">
         <v>None</v>
@@ -481,21 +481,21 @@
         <v>1</v>
       </c>
       <c r="M2">
-        <v>85.5</v>
+        <v>0</v>
       </c>
       <c r="N2" t="str">
-        <v>High</v>
+        <v>low</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Meenakshi Boutique</v>
+        <v>Lead Priority Score 1</v>
       </c>
       <c r="B3" t="str">
-        <v>+91 97890 12345</v>
+        <v>9840000001</v>
       </c>
       <c r="C3" t="str">
-        <v>info@meenakshiboutique.in</v>
+        <v>score1@example.com</v>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -504,13 +504,13 @@
         <v>Boutique</v>
       </c>
       <c r="F3" t="str">
-        <v>42, Arcot Road, Vellore, Tamil Nadu 632009</v>
+        <v>101 Test St, Vellore</v>
       </c>
       <c r="G3">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
       <c r="H3">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="I3" t="b">
         <v>0</v>
@@ -519,42 +519,42 @@
         <v>1</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3">
-        <v>92</v>
+        <v>1</v>
       </c>
       <c r="N3" t="str">
-        <v>High</v>
+        <v>cool</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Anand Dresses</v>
+        <v>Lead Priority Score 1.5</v>
       </c>
       <c r="B4" t="str">
-        <v>0416 2223344</v>
+        <v>9840000002</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>score15@example.com</v>
       </c>
       <c r="D4" t="str">
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>Clothing store</v>
+        <v>Boutique</v>
       </c>
       <c r="F4" t="str">
-        <v>Shop 3, Main Bazaar, Vellore</v>
+        <v>102 Test St, Vellore</v>
       </c>
       <c r="G4">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
       <c r="H4">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I4" t="b">
         <v>0</v>
@@ -563,92 +563,92 @@
         <v>1</v>
       </c>
       <c r="K4" t="str">
-        <v>Tally</v>
+        <v>None</v>
       </c>
       <c r="L4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4">
-        <v>55</v>
+        <v>1.5</v>
       </c>
       <c r="N4" t="str">
-        <v>Medium</v>
+        <v>cool</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>St. Marys Matriculation School</v>
+        <v>Lead Priority Score 1.99</v>
       </c>
       <c r="B5" t="str">
-        <v>9443322110</v>
+        <v>9840000003</v>
       </c>
       <c r="C5" t="str">
-        <v>stmarys.vlr@gmail.com</v>
+        <v>score199@example.com</v>
       </c>
       <c r="D5" t="str">
-        <v>https://stmarysschool.edu.in</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>School</v>
+        <v>Boutique</v>
       </c>
       <c r="F5" t="str">
-        <v>Katpadi Road, Vellore, Tamil Nadu 632007</v>
+        <v>103 Test St, Vellore</v>
       </c>
       <c r="G5">
-        <v>4.8</v>
+        <v>4.3</v>
       </c>
       <c r="H5">
-        <v>210</v>
+        <v>25</v>
       </c>
       <c r="I5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="str">
-        <v>Custom</v>
+        <v>None</v>
       </c>
       <c r="L5" t="b">
         <v>1</v>
       </c>
       <c r="M5">
-        <v>95</v>
+        <v>1.99</v>
       </c>
       <c r="N5" t="str">
-        <v>High</v>
+        <v>cool</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Vellore Vidhyashram</v>
+        <v>Lead Priority Score 2</v>
       </c>
       <c r="B6" t="str">
-        <v>087788 58303</v>
+        <v>9840000004</v>
       </c>
       <c r="C6" t="str">
-        <v>admissions@vvschool.ac.in</v>
+        <v>score2@example.com</v>
       </c>
       <c r="D6" t="str">
-        <v>https://vvschool.ac.in</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>School</v>
+        <v>Boutique</v>
       </c>
       <c r="F6" t="str">
-        <v>Sathuvachari, Vellore 632009</v>
+        <v>104 Test St, Vellore</v>
       </c>
       <c r="G6">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="H6">
-        <v>88</v>
+        <v>30</v>
       </c>
       <c r="I6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="str">
         <v>None</v>
@@ -657,21 +657,21 @@
         <v>1</v>
       </c>
       <c r="M6">
-        <v>88</v>
+        <v>2</v>
       </c>
       <c r="N6" t="str">
-        <v>High</v>
+        <v>cool</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Meenakshi Designer Studio</v>
+        <v>Lead Priority Score 3</v>
       </c>
       <c r="B7" t="str">
-        <v>9789012345</v>
+        <v>9840000005</v>
       </c>
       <c r="C7" t="str">
-        <v>studio@meenakshi.in</v>
+        <v>score3@example.com</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -680,13 +680,13 @@
         <v>Boutique</v>
       </c>
       <c r="F7" t="str">
-        <v>42 Arcot Road, 2nd floor, Vellore</v>
+        <v>105 Test St, Vellore</v>
       </c>
       <c r="G7">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="H7">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="I7" t="b">
         <v>0</v>
@@ -695,42 +695,42 @@
         <v>1</v>
       </c>
       <c r="K7" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L7" t="b">
         <v>1</v>
       </c>
       <c r="M7">
-        <v>70</v>
+        <v>3</v>
       </c>
       <c r="N7" t="str">
-        <v>Medium</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Modern Tailors &amp; Fabrics</v>
+        <v>Lead Priority Score 3.99</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>9840000006</v>
       </c>
       <c r="C8" t="str">
-        <v>moderntailors@yahoo.com</v>
+        <v>score399@example.com</v>
       </c>
       <c r="D8" t="str">
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Tailor</v>
+        <v>Boutique</v>
       </c>
       <c r="F8" t="str">
-        <v>10 Officer Line, Vellore</v>
+        <v>106 Test St, Vellore</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="H8">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="I8" t="b">
         <v>0</v>
@@ -739,174 +739,174 @@
         <v>1</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8">
-        <v>40</v>
+        <v>3.99</v>
       </c>
       <c r="N8" t="str">
-        <v>Low</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Royal Bridal Studio</v>
+        <v>Lead Priority Score 4</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>9840000007</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>score4@example.com</v>
       </c>
       <c r="D9" t="str">
-        <v>https://royalbridal.in</v>
+        <v/>
       </c>
       <c r="E9" t="str">
-        <v>Bridal shop</v>
+        <v>Boutique</v>
       </c>
       <c r="F9" t="str">
-        <v>Officers Line, Anna Salai, Vellore</v>
+        <v>107 Test St, Vellore</v>
       </c>
       <c r="G9">
         <v>4.7</v>
       </c>
       <c r="H9">
-        <v>65</v>
+        <v>45</v>
       </c>
       <c r="I9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="str">
-        <v>Zoho</v>
+        <v>None</v>
       </c>
       <c r="L9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="N9" t="str">
-        <v>Medium</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Krishna Silks Outlet</v>
+        <v>Lead Priority Score 5</v>
       </c>
       <c r="B10" t="str">
-        <v>+919840123456</v>
+        <v>9840000008</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>score5@example.com</v>
       </c>
       <c r="D10" t="str">
         <v/>
       </c>
       <c r="E10" t="str">
-        <v>Clothing store</v>
+        <v>Boutique</v>
       </c>
       <c r="F10" t="str">
-        <v>Gandhi Road Branch, Vellore</v>
+        <v>108 Test St, Vellore</v>
       </c>
       <c r="G10">
-        <v>4.1</v>
+        <v>4.8</v>
       </c>
       <c r="H10">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="N10" t="str">
-        <v>Low</v>
+        <v>hot</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Green Valley International School</v>
+        <v>Lead Blank Score Warm</v>
       </c>
       <c r="B11" t="str">
-        <v>9944556677</v>
+        <v>9840000009</v>
       </c>
       <c r="C11" t="str">
-        <v>principal@greenvalley.org</v>
+        <v>blankwarm@example.com</v>
       </c>
       <c r="D11" t="str">
-        <v>https://greenvalleyschool.org</v>
+        <v/>
       </c>
       <c r="E11" t="str">
-        <v>School</v>
+        <v>Boutique</v>
       </c>
       <c r="F11" t="str">
-        <v>Bagayam, Vellore, Tamil Nadu 632002</v>
+        <v>109 Test St, Vellore</v>
       </c>
       <c r="G11">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="H11">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="I11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" t="str">
-        <v>Tally</v>
+        <v>None</v>
       </c>
       <c r="L11" t="b">
         <v>1</v>
       </c>
-      <c r="M11">
-        <v>82</v>
+      <c r="M11" t="str">
+        <v/>
       </c>
       <c r="N11" t="str">
-        <v>High</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Kavitha Sarees &amp; Readymades</v>
+        <v>Lead Blank Score Hot</v>
       </c>
       <c r="B12" t="str">
-        <v>9442188776</v>
+        <v>9840000010</v>
       </c>
       <c r="C12" t="str">
-        <v>kavithasarees@gmail.com</v>
+        <v>blankhot@example.com</v>
       </c>
       <c r="D12" t="str">
         <v/>
       </c>
       <c r="E12" t="str">
-        <v>Saree shop</v>
+        <v>Boutique</v>
       </c>
       <c r="F12" t="str">
-        <v>Bazaar Street, Gudiyattam, Vellore 632602</v>
+        <v>110 Test St, Vellore</v>
       </c>
       <c r="G12">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="H12">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="I12" t="b">
         <v>0</v>
@@ -915,42 +915,42 @@
         <v>1</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L12" t="b">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>65</v>
+        <v>1</v>
+      </c>
+      <c r="M12" t="str">
+        <v/>
       </c>
       <c r="N12" t="str">
-        <v>Medium</v>
+        <v>hot</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Little Flower Nursery &amp; Primary School</v>
+        <v>Lead Text Score NA</v>
       </c>
       <c r="B13" t="str">
-        <v>9842345678</v>
+        <v>9840000011</v>
       </c>
       <c r="C13" t="str">
-        <v>lfps.vellore@gmail.com</v>
+        <v>scorena@example.com</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
       <c r="E13" t="str">
-        <v>Primary school</v>
+        <v>Boutique</v>
       </c>
       <c r="F13" t="str">
-        <v>Thorapadi, Vellore 632002</v>
+        <v>111 Test St, Vellore</v>
       </c>
       <c r="G13">
-        <v>4.1</v>
+        <v>3.9</v>
       </c>
       <c r="H13">
-        <v>52</v>
+        <v>8</v>
       </c>
       <c r="I13" t="b">
         <v>0</v>
@@ -959,130 +959,130 @@
         <v>1</v>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L13" t="b">
         <v>1</v>
       </c>
-      <c r="M13">
-        <v>75</v>
+      <c r="M13" t="str">
+        <v>n/a</v>
       </c>
       <c r="N13" t="str">
-        <v>Medium</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Trends &amp; Fashions Boutique</v>
+        <v>Lead Score Seven Out Of Range</v>
       </c>
       <c r="B14" t="str">
-        <v>9790112233</v>
+        <v>9840000012</v>
       </c>
       <c r="C14" t="str">
-        <v>orders@trendsfashions.com</v>
+        <v>score7@example.com</v>
       </c>
       <c r="D14" t="str">
-        <v>https://trendsfashions.com</v>
+        <v/>
       </c>
       <c r="E14" t="str">
-        <v>Women clothing store</v>
+        <v>Boutique</v>
       </c>
       <c r="F14" t="str">
-        <v>Phase 2, Sathuvachari, Vellore</v>
+        <v>112 Test St, Vellore</v>
       </c>
       <c r="G14">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
       <c r="H14">
-        <v>94</v>
+        <v>14</v>
       </c>
       <c r="I14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="str">
-        <v>Shopify</v>
+        <v>None</v>
       </c>
       <c r="L14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M14">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="N14" t="str">
-        <v>Medium</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Seventh Day Adventist High School</v>
+        <v>Sri Krishna Silks</v>
       </c>
       <c r="B15" t="str">
-        <v>9443124578</v>
+        <v>9840123456</v>
       </c>
       <c r="C15" t="str">
-        <v>sda.school@rediffmail.com</v>
+        <v>contact@krishnasilks.com</v>
       </c>
       <c r="D15" t="str">
-        <v/>
+        <v>https://krishnasilks.com</v>
       </c>
       <c r="E15" t="str">
-        <v>High school</v>
+        <v>Silk store</v>
       </c>
       <c r="F15" t="str">
-        <v>Otteri Road, Vellore 632002</v>
+        <v>14, Gandhi Road, Vellore, Tamil Nadu 632004</v>
       </c>
       <c r="G15">
-        <v>4.3</v>
+        <v>4.5</v>
       </c>
       <c r="H15">
-        <v>76</v>
+        <v>120</v>
       </c>
       <c r="I15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K15" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L15" t="b">
         <v>1</v>
       </c>
       <c r="M15">
-        <v>84</v>
+        <v>4.5</v>
       </c>
       <c r="N15" t="str">
-        <v>High</v>
+        <v>hot</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Vaishnavi Aari &amp; Embroidery</v>
+        <v>Meenakshi Boutique</v>
       </c>
       <c r="B16" t="str">
-        <v>8056712389</v>
+        <v>+91 97890 12345</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>info@meenakshiboutique.in</v>
       </c>
       <c r="D16" t="str">
         <v/>
       </c>
       <c r="E16" t="str">
-        <v>Embroidery service</v>
+        <v>Boutique</v>
       </c>
       <c r="F16" t="str">
-        <v>Kosapet, Vellore 632001</v>
+        <v>42, Arcot Road, Vellore, Tamil Nadu 632009</v>
       </c>
       <c r="G16">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="H16">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I16" t="b">
         <v>0</v>
@@ -1097,124 +1097,124 @@
         <v>0</v>
       </c>
       <c r="M16">
-        <v>68</v>
+        <v>4.2</v>
       </c>
       <c r="N16" t="str">
-        <v>Medium</v>
+        <v>hot</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Adarsh Vidyalaya Matriculation Higher Secondary</v>
+        <v>Anand Dresses</v>
       </c>
       <c r="B17" t="str">
-        <v>9841029384</v>
+        <v>0416 2223344</v>
       </c>
       <c r="C17" t="str">
-        <v>adarsh.vellore@yahoo.co.in</v>
+        <v/>
       </c>
       <c r="D17" t="str">
-        <v>https://adarshvidyalaya.in</v>
+        <v/>
       </c>
       <c r="E17" t="str">
-        <v>School</v>
+        <v>Clothing store</v>
       </c>
       <c r="F17" t="str">
-        <v>Katpadi, Vellore 632014</v>
+        <v>Shop 3, Main Bazaar, Vellore</v>
       </c>
       <c r="G17">
-        <v>4.7</v>
+        <v>3.8</v>
       </c>
       <c r="H17">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="I17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K17" t="str">
-        <v>None</v>
+        <v>Tally</v>
       </c>
       <c r="L17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17">
-        <v>91</v>
+        <v>2.5</v>
       </c>
       <c r="N17" t="str">
-        <v>High</v>
+        <v>cool</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Aura Women Boutique &amp; Spa</v>
+        <v>St. Marys Matriculation School</v>
       </c>
       <c r="B18" t="str">
-        <v>9176543210</v>
+        <v>9443322110</v>
       </c>
       <c r="C18" t="str">
-        <v>auraspa@gmail.com</v>
+        <v>stmarys.vlr@gmail.com</v>
       </c>
       <c r="D18" t="str">
-        <v/>
+        <v>https://stmarysschool.edu.in</v>
       </c>
       <c r="E18" t="str">
-        <v>Beauty parlour</v>
+        <v>School</v>
       </c>
       <c r="F18" t="str">
-        <v>Gandhi Nagar, Katpadi, Vellore</v>
+        <v>Katpadi Road, Vellore, Tamil Nadu 632007</v>
       </c>
       <c r="G18">
-        <v>4.2</v>
+        <v>4.8</v>
       </c>
       <c r="H18">
-        <v>61</v>
+        <v>210</v>
       </c>
       <c r="I18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="str">
-        <v/>
+        <v>Custom</v>
       </c>
       <c r="L18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18">
-        <v>72</v>
+        <v>4.8</v>
       </c>
       <c r="N18" t="str">
-        <v>Medium</v>
+        <v>hot</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sparkle Kidz Pre School</v>
+        <v>Vellore Vidhyashram</v>
       </c>
       <c r="B19" t="str">
-        <v>9629112244</v>
+        <v>087788 58303</v>
       </c>
       <c r="C19" t="str">
-        <v>hello@sparklekidz.com</v>
+        <v>admissions@vvschool.ac.in</v>
       </c>
       <c r="D19" t="str">
-        <v>https://sparklekidz.com</v>
+        <v>https://vvschool.ac.in</v>
       </c>
       <c r="E19" t="str">
-        <v>Preschool</v>
+        <v>School</v>
       </c>
       <c r="F19" t="str">
-        <v>Kangeyanallur Road, Katpadi</v>
+        <v>Sathuvachari, Vellore 632009</v>
       </c>
       <c r="G19">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="H19">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
@@ -1223,42 +1223,42 @@
         <v>0</v>
       </c>
       <c r="K19" t="str">
-        <v/>
+        <v>None</v>
       </c>
       <c r="L19" t="b">
         <v>1</v>
       </c>
       <c r="M19">
-        <v>86</v>
+        <v>4</v>
       </c>
       <c r="N19" t="str">
-        <v>High</v>
+        <v>warm</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Style Zone Mens &amp; Kids Wear</v>
+        <v>Modern Tailors &amp; Fabrics</v>
       </c>
       <c r="B20" t="str">
-        <v>9443765432</v>
+        <v/>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>moderntailors@yahoo.com</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
       <c r="E20" t="str">
-        <v>Clothing store</v>
+        <v>Tailor</v>
       </c>
       <c r="F20" t="str">
-        <v>Near Old Bus Stand, Vellore</v>
+        <v>10 Officer Line, Vellore</v>
       </c>
       <c r="G20">
-        <v>3.7</v>
+        <v>4</v>
       </c>
       <c r="H20">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I20" t="b">
         <v>0</v>
@@ -1273,54 +1273,54 @@
         <v>0</v>
       </c>
       <c r="M20">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="N20" t="str">
-        <v>Low</v>
+        <v>low</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Saraswathi Vidyalaya School</v>
+        <v>Royal Bridal Studio</v>
       </c>
       <c r="B21" t="str">
-        <v>9840987654</v>
+        <v/>
       </c>
       <c r="C21" t="str">
-        <v>svschool@gmail.com</v>
+        <v/>
       </c>
       <c r="D21" t="str">
-        <v/>
+        <v>https://royalbridal.in</v>
       </c>
       <c r="E21" t="str">
-        <v>School</v>
+        <v>Bridal shop</v>
       </c>
       <c r="F21" t="str">
-        <v>Kaspa, Vellore 632001</v>
+        <v>Officers Line, Anna Salai, Vellore</v>
       </c>
       <c r="G21">
-        <v>4</v>
+        <v>4.7</v>
       </c>
       <c r="H21">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K21" t="str">
-        <v>None</v>
+        <v>Zoho</v>
       </c>
       <c r="L21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21">
-        <v>79</v>
+        <v>3.2</v>
       </c>
       <c r="N21" t="str">
-        <v>Medium</v>
+        <v>warm</v>
       </c>
     </row>
   </sheetData>

</xml_diff>